<commit_message>
test(cart): add shopping cart automation suite
</commit_message>
<xml_diff>
--- a/docs/manual-testing/AEQA_Manual_Test_Suite.xlsx
+++ b/docs/manual-testing/AEQA_Manual_Test_Suite.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Documents/automation-exercise-qa/docs/manual-testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FEB740-CAFD-4941-9D54-E87AAD44F410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{353E6B5C-A003-9740-9BED-214811481F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14480" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14480" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Overview" sheetId="1" r:id="rId1"/>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="E8" s="1">
         <f>COUNTIF('01_Authentication'!$N$2:$N$200,"Not Run")+COUNTIF('02_Products'!$N$2:$N$200,"Not Run")+COUNTIF('03_Cart'!$N$2:$N$200,"Not Run")+COUNTIF('04_Checkout'!$N$2:$N$200,"Not Run")+COUNTIF('05_Support'!$N$2:$N$200,"Not Run")+COUNTIF('06_Navigation'!$N$2:$N$200,"Not Run")+COUNTIF('07_API'!$N$2:$N$200,"Not Run")</f>
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -4164,11 +4164,11 @@
       </c>
       <c r="H15" s="9">
         <f>COUNTIF('03_Cart'!$N$2:$N$200,"Not Run")</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I15" s="9">
         <f>COUNTIF('03_Cart'!$N$2:$N$200,"Pass")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J15" s="9">
         <f>COUNTIF('03_Cart'!$N$2:$N$200,"Fail")</f>
@@ -11475,7 +11475,7 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>91</v>
@@ -11541,7 +11541,7 @@
       </c>
       <c r="M3" s="5"/>
       <c r="N3" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O3" s="5" t="s">
         <v>91</v>
@@ -11607,7 +11607,7 @@
       </c>
       <c r="M4" s="5"/>
       <c r="N4" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O4" s="5" t="s">
         <v>114</v>
@@ -11673,7 +11673,7 @@
       </c>
       <c r="M5" s="5"/>
       <c r="N5" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>91</v>
@@ -11739,7 +11739,7 @@
       </c>
       <c r="M6" s="5"/>
       <c r="N6" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>114</v>
@@ -11805,7 +11805,7 @@
       </c>
       <c r="M7" s="5"/>
       <c r="N7" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O7" s="5" t="s">
         <v>91</v>
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M8" s="5"/>
       <c r="N8" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O8" s="5" t="s">
         <v>114</v>
@@ -11937,7 +11937,7 @@
       </c>
       <c r="M9" s="5"/>
       <c r="N9" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O9" s="5" t="s">
         <v>91</v>

</xml_diff>

<commit_message>
test(checkout): add checkout automation suite
</commit_message>
<xml_diff>
--- a/docs/manual-testing/AEQA_Manual_Test_Suite.xlsx
+++ b/docs/manual-testing/AEQA_Manual_Test_Suite.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Documents/automation-exercise-qa/docs/manual-testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{353E6B5C-A003-9740-9BED-214811481F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E5F3C3-C299-3848-8C26-D8DCA23D3559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14480" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14440" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Overview" sheetId="1" r:id="rId1"/>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="E8" s="1">
         <f>COUNTIF('01_Authentication'!$N$2:$N$200,"Not Run")+COUNTIF('02_Products'!$N$2:$N$200,"Not Run")+COUNTIF('03_Cart'!$N$2:$N$200,"Not Run")+COUNTIF('04_Checkout'!$N$2:$N$200,"Not Run")+COUNTIF('05_Support'!$N$2:$N$200,"Not Run")+COUNTIF('06_Navigation'!$N$2:$N$200,"Not Run")+COUNTIF('07_API'!$N$2:$N$200,"Not Run")</f>
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -4207,11 +4207,11 @@
       </c>
       <c r="H16" s="9">
         <f>COUNTIF('04_Checkout'!$N$2:$N$200,"Not Run")</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I16" s="9">
         <f>COUNTIF('04_Checkout'!$N$2:$N$200,"Pass")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J16" s="9">
         <f>COUNTIF('04_Checkout'!$N$2:$N$200,"Fail")</f>
@@ -4250,11 +4250,11 @@
       </c>
       <c r="H17" s="9">
         <f>COUNTIF('05_Support'!$N$2:$N$200,"Not Run")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I17" s="9">
         <f>COUNTIF('05_Support'!$N$2:$N$200,"Pass")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J17" s="9">
         <f>COUNTIF('05_Support'!$N$2:$N$200,"Fail")</f>
@@ -13136,7 +13136,7 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>91</v>
@@ -13202,7 +13202,7 @@
       </c>
       <c r="M3" s="5"/>
       <c r="N3" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O3" s="5" t="s">
         <v>91</v>
@@ -13268,7 +13268,7 @@
       </c>
       <c r="M4" s="5"/>
       <c r="N4" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O4" s="5" t="s">
         <v>91</v>
@@ -13334,7 +13334,7 @@
       </c>
       <c r="M5" s="5"/>
       <c r="N5" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>91</v>
@@ -13400,7 +13400,7 @@
       </c>
       <c r="M6" s="5"/>
       <c r="N6" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>91</v>
@@ -13466,7 +13466,7 @@
       </c>
       <c r="M7" s="5"/>
       <c r="N7" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O7" s="5" t="s">
         <v>114</v>
@@ -13532,7 +13532,7 @@
       </c>
       <c r="M8" s="5"/>
       <c r="N8" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O8" s="5" t="s">
         <v>91</v>
@@ -13598,7 +13598,7 @@
       </c>
       <c r="M9" s="5"/>
       <c r="N9" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O9" s="5" t="s">
         <v>114</v>
@@ -14797,7 +14797,7 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>114</v>
@@ -14862,8 +14862,8 @@
         <v>436</v>
       </c>
       <c r="M3" s="5"/>
-      <c r="N3" s="5" t="s">
-        <v>24</v>
+      <c r="N3" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O3" s="5" t="s">
         <v>273</v>
@@ -14928,8 +14928,8 @@
         <v>272</v>
       </c>
       <c r="M4" s="5"/>
-      <c r="N4" s="5" t="s">
-        <v>24</v>
+      <c r="N4" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O4" s="5" t="s">
         <v>273</v>
@@ -14994,8 +14994,8 @@
         <v>448</v>
       </c>
       <c r="M5" s="5"/>
-      <c r="N5" s="5" t="s">
-        <v>24</v>
+      <c r="N5" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>114</v>
@@ -15060,8 +15060,8 @@
         <v>448</v>
       </c>
       <c r="M6" s="5"/>
-      <c r="N6" s="5" t="s">
-        <v>24</v>
+      <c r="N6" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>114</v>
@@ -15126,8 +15126,8 @@
         <v>460</v>
       </c>
       <c r="M7" s="5"/>
-      <c r="N7" s="5" t="s">
-        <v>24</v>
+      <c r="N7" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O7" s="5" t="s">
         <v>273</v>

</xml_diff>

<commit_message>
test(navigation): add navigation automation suite
</commit_message>
<xml_diff>
--- a/docs/manual-testing/AEQA_Manual_Test_Suite.xlsx
+++ b/docs/manual-testing/AEQA_Manual_Test_Suite.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Documents/automation-exercise-qa/docs/manual-testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E5F3C3-C299-3848-8C26-D8DCA23D3559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C1D771-DAB5-3547-BD6B-1DACB9CFCDE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14440" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="14440" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Overview" sheetId="1" r:id="rId1"/>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="E8" s="1">
         <f>COUNTIF('01_Authentication'!$N$2:$N$200,"Not Run")+COUNTIF('02_Products'!$N$2:$N$200,"Not Run")+COUNTIF('03_Cart'!$N$2:$N$200,"Not Run")+COUNTIF('04_Checkout'!$N$2:$N$200,"Not Run")+COUNTIF('05_Support'!$N$2:$N$200,"Not Run")+COUNTIF('06_Navigation'!$N$2:$N$200,"Not Run")+COUNTIF('07_API'!$N$2:$N$200,"Not Run")</f>
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -4293,11 +4293,11 @@
       </c>
       <c r="H18" s="9">
         <f>COUNTIF('06_Navigation'!$N$2:$N$200,"Not Run")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I18" s="9">
         <f>COUNTIF('06_Navigation'!$N$2:$N$200,"Pass")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J18" s="9">
         <f>COUNTIF('06_Navigation'!$N$2:$N$200,"Fail")</f>
@@ -4336,11 +4336,11 @@
       </c>
       <c r="H19" s="9">
         <f>COUNTIF('07_API'!$N$2:$N$200,"Not Run")</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="I19" s="9">
         <f>COUNTIF('07_API'!$N$2:$N$200,"Pass")</f>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J19" s="9">
         <f>COUNTIF('07_API'!$N$2:$N$200,"Fail")</f>
@@ -16326,7 +16326,7 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>114</v>
@@ -16391,8 +16391,8 @@
         <v>475</v>
       </c>
       <c r="M3" s="5"/>
-      <c r="N3" s="5" t="s">
-        <v>24</v>
+      <c r="N3" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O3" s="5" t="s">
         <v>273</v>
@@ -16455,8 +16455,8 @@
         <v>483</v>
       </c>
       <c r="M4" s="5"/>
-      <c r="N4" s="5" t="s">
-        <v>24</v>
+      <c r="N4" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O4" s="5" t="s">
         <v>273</v>
@@ -16521,8 +16521,8 @@
         <v>491</v>
       </c>
       <c r="M5" s="5"/>
-      <c r="N5" s="5" t="s">
-        <v>24</v>
+      <c r="N5" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>273</v>
@@ -16585,8 +16585,8 @@
         <v>498</v>
       </c>
       <c r="M6" s="5"/>
-      <c r="N6" s="5" t="s">
-        <v>24</v>
+      <c r="N6" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>273</v>
@@ -17783,7 +17783,7 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>91</v>
@@ -17848,8 +17848,8 @@
         <v>516</v>
       </c>
       <c r="M3" s="5"/>
-      <c r="N3" s="5" t="s">
-        <v>24</v>
+      <c r="N3" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O3" s="5" t="s">
         <v>91</v>
@@ -17914,8 +17914,8 @@
         <v>525</v>
       </c>
       <c r="M4" s="5"/>
-      <c r="N4" s="5" t="s">
-        <v>24</v>
+      <c r="N4" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O4" s="5" t="s">
         <v>91</v>
@@ -17980,8 +17980,8 @@
         <v>516</v>
       </c>
       <c r="M5" s="5"/>
-      <c r="N5" s="5" t="s">
-        <v>24</v>
+      <c r="N5" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>91</v>
@@ -18046,8 +18046,8 @@
         <v>539</v>
       </c>
       <c r="M6" s="5"/>
-      <c r="N6" s="5" t="s">
-        <v>24</v>
+      <c r="N6" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>91</v>
@@ -18112,8 +18112,8 @@
         <v>546</v>
       </c>
       <c r="M7" s="5"/>
-      <c r="N7" s="5" t="s">
-        <v>24</v>
+      <c r="N7" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O7" s="5" t="s">
         <v>91</v>
@@ -18178,8 +18178,8 @@
         <v>555</v>
       </c>
       <c r="M8" s="5"/>
-      <c r="N8" s="5" t="s">
-        <v>24</v>
+      <c r="N8" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O8" s="5" t="s">
         <v>91</v>
@@ -18244,8 +18244,8 @@
         <v>561</v>
       </c>
       <c r="M9" s="5"/>
-      <c r="N9" s="5" t="s">
-        <v>24</v>
+      <c r="N9" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O9" s="5" t="s">
         <v>91</v>
@@ -18310,8 +18310,8 @@
         <v>516</v>
       </c>
       <c r="M10" s="5"/>
-      <c r="N10" s="5" t="s">
-        <v>24</v>
+      <c r="N10" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O10" s="5" t="s">
         <v>91</v>
@@ -18376,8 +18376,8 @@
         <v>574</v>
       </c>
       <c r="M11" s="5"/>
-      <c r="N11" s="5" t="s">
-        <v>24</v>
+      <c r="N11" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O11" s="5" t="s">
         <v>91</v>
@@ -18442,8 +18442,8 @@
         <v>583</v>
       </c>
       <c r="M12" s="5"/>
-      <c r="N12" s="5" t="s">
-        <v>24</v>
+      <c r="N12" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O12" s="5" t="s">
         <v>91</v>
@@ -18508,8 +18508,8 @@
         <v>590</v>
       </c>
       <c r="M13" s="5"/>
-      <c r="N13" s="5" t="s">
-        <v>24</v>
+      <c r="N13" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O13" s="5" t="s">
         <v>91</v>
@@ -18574,8 +18574,8 @@
         <v>596</v>
       </c>
       <c r="M14" s="5"/>
-      <c r="N14" s="5" t="s">
-        <v>24</v>
+      <c r="N14" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O14" s="5" t="s">
         <v>91</v>
@@ -18640,8 +18640,8 @@
         <v>602</v>
       </c>
       <c r="M15" s="5"/>
-      <c r="N15" s="5" t="s">
-        <v>24</v>
+      <c r="N15" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="O15" s="5" t="s">
         <v>91</v>

</xml_diff>